<commit_message>
feat: install image detect module
</commit_message>
<xml_diff>
--- a/assets/example1/example1.xlsx
+++ b/assets/example1/example1.xlsx
@@ -1664,7 +1664,7 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>生成時間：2025-06-20 17:09:02 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
+          <t>生成時間：2025-06-21 07:13:56 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>生成時間：2025-06-20 17:09:03 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
+          <t>生成時間：2025-06-21 07:13:56 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>生成時間：2025-06-20 17:09:03 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
+          <t>生成時間：2025-06-21 07:13:56 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>生成時間：2025-06-20 17:09:03 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
+          <t>生成時間：2025-06-21 07:13:56 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>生成時間：2025-06-20 17:09:03 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
+          <t>生成時間：2025-06-21 07:13:57 | 圖示模式：圖文混合模式 | 圖形功能：啟用</t>
         </is>
       </c>
     </row>

</xml_diff>